<commit_message>
Actualisation du tableau de synthèse des compétences
</commit_message>
<xml_diff>
--- a/tableau-synthese.xlsx
+++ b/tableau-synthese.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julien\Documents\BTS SIO Iris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68FA4F9B-B65C-4A0F-8852-FD7EB3592D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB9C48E-E88F-49BF-9E45-4724DE3F596A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -762,15 +762,39 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -802,30 +826,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1210,56 +1210,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="H1" s="26"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="44" t="s">
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="39"/>
-      <c r="H3" s="45"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="32"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="43"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="12" t="s">
         <v>2</v>
       </c>
@@ -1271,22 +1271,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="37"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="45"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="41" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1309,8 +1309,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25"/>
-      <c r="B7" s="34"/>
+      <c r="A7" s="34"/>
+      <c r="B7" s="42"/>
       <c r="C7" s="19" t="s">
         <v>13</v>
       </c>
@@ -1366,16 +1366,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="37"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1836,16 +1836,16 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="32"/>
+      <c r="B18" s="39"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="40"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1887,8 +1887,8 @@
         <v>36</v>
       </c>
       <c r="B19" s="8"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
       <c r="G19" s="14"/>
@@ -1934,10 +1934,10 @@
         <v>37</v>
       </c>
       <c r="B20" s="8"/>
-      <c r="C20" s="14"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="21"/>
       <c r="G20" s="14"/>
       <c r="H20" s="15"/>
       <c r="I20"/>
@@ -1984,9 +1984,9 @@
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="21"/>
       <c r="G21" s="14"/>
-      <c r="H21" s="15"/>
+      <c r="H21" s="22"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -2204,16 +2204,16 @@
       <c r="AQ25"/>
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A26" s="30" t="s">
+      <c r="A26" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="31"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="31"/>
-      <c r="H26" s="32"/>
+      <c r="B26" s="39"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="40"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2255,10 +2255,10 @@
         <v>40</v>
       </c>
       <c r="B27" s="8"/>
-      <c r="C27" s="14"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="14"/>
       <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
+      <c r="F27" s="21"/>
       <c r="G27" s="14"/>
       <c r="H27" s="15"/>
       <c r="I27"/>
@@ -2303,8 +2303,8 @@
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
       <c r="F28" s="14"/>
       <c r="G28" s="14"/>
       <c r="H28" s="15"/>
@@ -2349,10 +2349,10 @@
         <v>41</v>
       </c>
       <c r="B29" s="8"/>
-      <c r="C29" s="14"/>
+      <c r="C29" s="21"/>
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
+      <c r="F29" s="21"/>
       <c r="G29" s="14"/>
       <c r="H29" s="15"/>
       <c r="I29"/>
@@ -2397,9 +2397,9 @@
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
+      <c r="D30" s="21"/>
       <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
+      <c r="F30" s="21"/>
       <c r="G30" s="14"/>
       <c r="H30" s="15"/>
       <c r="I30"/>
@@ -2443,10 +2443,10 @@
         <v>43</v>
       </c>
       <c r="B31" s="8"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
       <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
+      <c r="F31" s="21"/>
       <c r="G31" s="14"/>
       <c r="H31" s="15"/>
       <c r="I31"/>
@@ -2668,11 +2668,6 @@
     <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2680,6 +2675,11 @@
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2691,14 +2691,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="665588ff-5dd3-431a-aaf4-bd4a76d54561">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8dfcfa40-b15b-4f0f-a13d-24527312d446" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2909,21 +2907,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="665588ff-5dd3-431a-aaf4-bd4a76d54561">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8dfcfa40-b15b-4f0f-a13d-24527312d446" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B48EC0E1-0992-4BEA-AB73-03077E430CDC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A9CD917-9C6C-4808-B3EB-08BF761FD3DB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="665588ff-5dd3-431a-aaf4-bd4a76d54561"/>
-    <ds:schemaRef ds:uri="8dfcfa40-b15b-4f0f-a13d-24527312d446"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2948,9 +2945,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A9CD917-9C6C-4808-B3EB-08BF761FD3DB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B48EC0E1-0992-4BEA-AB73-03077E430CDC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="665588ff-5dd3-431a-aaf4-bd4a76d54561"/>
+    <ds:schemaRef ds:uri="8dfcfa40-b15b-4f0f-a13d-24527312d446"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>